<commit_message>
Update panel B data and add flanking-regions note to panel C title
- Panel B now uses the updated plasmid workbook (bacteriocin module
  expanded to 4 genes, sheet name normalized).
- Panel C title now reads "mecA + ACME cassette (JE2) + flanking
  regions" to reflect the added flanking genes.
</commit_message>
<xml_diff>
--- a/figures/shap_heatmaps/data/N315_plasmid.xlsx
+++ b/figures/shap_heatmaps/data/N315_plasmid.xlsx
@@ -5,22 +5,22 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paultorrillo/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paultorrillo/Downloads/hunting_for_good_shaps/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C20207E2-191C-124C-921A-5A9EB5A517CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB5D9A79-0B52-8946-B970-075055675051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="1480" windowWidth="27240" windowHeight="15440"/>
+    <workbookView xWindow="1980" yWindow="2500" windowWidth="26440" windowHeight="14440"/>
   </bookViews>
   <sheets>
-    <sheet name="selected_gene_directional_shap_" sheetId="1" r:id="rId1"/>
+    <sheet name="selected_gene_directional_shap" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="63">
   <si>
     <t>row_gene_idx</t>
   </si>
@@ -205,7 +205,7 @@
     <t>Arsenical resistance</t>
   </si>
   <si>
-    <t>Bacteriocin module</t>
+    <t>Putative bacteriocin module</t>
   </si>
   <si>
     <t>plamid recombination</t>
@@ -692,9 +692,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1053,8 +1052,9 @@
   <dimension ref="A1:AC27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="70.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.2">
@@ -1160,79 +1160,79 @@
         <v>29</v>
       </c>
       <c r="E2">
-        <v>-0.18103820000000001</v>
+        <v>-0.1870146</v>
       </c>
       <c r="F2">
-        <v>-0.5005153</v>
+        <v>-0.53131019999999995</v>
       </c>
       <c r="G2">
-        <v>-0.17952099999999999</v>
+        <v>-0.19250639999999999</v>
       </c>
       <c r="H2">
-        <v>-0.1619458</v>
+        <v>-0.17481250000000001</v>
       </c>
       <c r="I2">
-        <v>-0.18053910000000001</v>
+        <v>-0.19086130000000001</v>
       </c>
       <c r="J2">
-        <v>-5.76558E-2</v>
+        <v>-5.5665800000000001E-2</v>
       </c>
       <c r="K2">
-        <v>-0.2461158</v>
+        <v>-0.26151819999999998</v>
       </c>
       <c r="L2">
-        <v>-0.22863919999999999</v>
+        <v>-0.23322219999999999</v>
       </c>
       <c r="M2">
-        <v>-4.9415800000000003E-2</v>
+        <v>-5.4107799999999998E-2</v>
       </c>
       <c r="N2">
-        <v>-0.13588919999999999</v>
+        <v>-0.1560975</v>
       </c>
       <c r="O2">
-        <v>-5.9848999999999999E-2</v>
+        <v>-6.5645899999999993E-2</v>
       </c>
       <c r="P2">
-        <v>-5.3970700000000003E-2</v>
+        <v>-6.3030000000000003E-2</v>
       </c>
       <c r="Q2">
-        <v>-7.0525199999999996E-2</v>
+        <v>-7.5407699999999994E-2</v>
       </c>
       <c r="R2">
-        <v>-0.14605319999999999</v>
+        <v>-0.15903610000000001</v>
       </c>
       <c r="S2">
-        <v>-0.12928899999999999</v>
+        <v>-0.13848269999999999</v>
       </c>
       <c r="T2">
-        <v>-0.1231718</v>
+        <v>-0.13098309999999999</v>
       </c>
       <c r="U2">
-        <v>0.1223154</v>
+        <v>0.13680310000000001</v>
       </c>
       <c r="V2">
-        <v>-6.1445E-2</v>
+        <v>-5.75846E-2</v>
       </c>
       <c r="W2">
-        <v>-6.2283600000000001E-2</v>
+        <v>-6.2091500000000001E-2</v>
       </c>
       <c r="X2">
-        <v>-5.6048000000000001E-2</v>
+        <v>-5.4466100000000003E-2</v>
       </c>
       <c r="Y2">
-        <v>-0.1348453</v>
+        <v>-0.14285030000000001</v>
       </c>
       <c r="Z2">
-        <v>-0.1153018</v>
+        <v>-0.1208993</v>
       </c>
       <c r="AA2">
-        <v>0.16885269999999999</v>
+        <v>0.18186820000000001</v>
       </c>
       <c r="AB2">
-        <v>0.13589019999999999</v>
+        <v>0.15091180000000001</v>
       </c>
       <c r="AC2">
-        <v>-0.1447474</v>
+        <v>-0.15373629999999999</v>
       </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.2">
@@ -1246,82 +1246,82 @@
         <v>30</v>
       </c>
       <c r="D3">
-        <v>8.4183999999999995E-3</v>
+        <v>1.08377E-2</v>
       </c>
       <c r="E3" t="s">
         <v>29</v>
       </c>
       <c r="F3">
-        <v>-0.57490490000000005</v>
+        <v>-0.62121389999999999</v>
       </c>
       <c r="G3">
-        <v>-7.8758999999999999E-3</v>
+        <v>-4.4822999999999998E-3</v>
       </c>
       <c r="H3">
-        <v>-8.9380500000000002E-2</v>
+        <v>-8.9878399999999997E-2</v>
       </c>
       <c r="I3">
-        <v>5.5223700000000001E-2</v>
+        <v>5.2301500000000001E-2</v>
       </c>
       <c r="J3">
-        <v>1.78058E-2</v>
+        <v>1.71924E-2</v>
       </c>
       <c r="K3">
-        <v>-9.0336899999999998E-2</v>
+        <v>-9.6641599999999994E-2</v>
       </c>
       <c r="L3">
-        <v>-0.136013</v>
+        <v>-0.14622959999999999</v>
       </c>
       <c r="M3">
-        <v>3.5616299999999997E-2</v>
+        <v>3.7205599999999998E-2</v>
       </c>
       <c r="N3">
-        <v>5.71592E-2</v>
+        <v>5.87786E-2</v>
       </c>
       <c r="O3">
-        <v>5.4199000000000001E-3</v>
+        <v>3.2355999999999999E-3</v>
       </c>
       <c r="P3">
-        <v>-1.55709E-2</v>
+        <v>-1.29176E-2</v>
       </c>
       <c r="Q3">
-        <v>-1.5026E-3</v>
+        <v>1.5540000000000001E-4</v>
       </c>
       <c r="R3">
-        <v>-0.26025530000000002</v>
+        <v>-0.28314460000000002</v>
       </c>
       <c r="S3">
-        <v>-0.23160800000000001</v>
+        <v>-0.2543125</v>
       </c>
       <c r="T3">
-        <v>-0.2455417</v>
+        <v>-0.26847949999999998</v>
       </c>
       <c r="U3">
-        <v>-0.1485416</v>
+        <v>-0.1696394</v>
       </c>
       <c r="V3">
-        <v>-0.1145322</v>
+        <v>-0.13786880000000001</v>
       </c>
       <c r="W3">
-        <v>-0.12854869999999999</v>
+        <v>-0.1463496</v>
       </c>
       <c r="X3">
-        <v>-0.12451089999999999</v>
+        <v>-0.1408867</v>
       </c>
       <c r="Y3">
-        <v>-0.28646120000000003</v>
+        <v>-0.31385859999999999</v>
       </c>
       <c r="Z3">
-        <v>-0.27957460000000001</v>
+        <v>-0.30475410000000003</v>
       </c>
       <c r="AA3">
-        <v>-0.17706269999999999</v>
+        <v>-0.19718630000000001</v>
       </c>
       <c r="AB3">
-        <v>-0.14265800000000001</v>
+        <v>-0.1640626</v>
       </c>
       <c r="AC3">
-        <v>0.13330739999999999</v>
+        <v>0.13965069999999999</v>
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.2">
@@ -1332,82 +1332,82 @@
         <v>31</v>
       </c>
       <c r="D4">
-        <v>9.03254E-2</v>
+        <v>9.1344999999999996E-2</v>
       </c>
       <c r="E4">
-        <v>-0.17128180000000001</v>
+        <v>-0.18602009999999999</v>
       </c>
       <c r="F4" t="s">
         <v>29</v>
       </c>
       <c r="G4">
-        <v>-4.9111799999999997E-2</v>
+        <v>-5.6388800000000003E-2</v>
       </c>
       <c r="H4">
-        <v>-6.15951E-2</v>
+        <v>-7.1436700000000006E-2</v>
       </c>
       <c r="I4">
-        <v>9.3079099999999998E-2</v>
+        <v>9.8721500000000004E-2</v>
       </c>
       <c r="J4">
-        <v>0.19262950000000001</v>
+        <v>0.20419989999999999</v>
       </c>
       <c r="K4">
-        <v>0.14556189999999999</v>
+        <v>0.15865699999999999</v>
       </c>
       <c r="L4">
-        <v>0.1845726</v>
+        <v>0.20164370000000001</v>
       </c>
       <c r="M4">
-        <v>8.5886299999999999E-2</v>
+        <v>8.86078E-2</v>
       </c>
       <c r="N4">
-        <v>-1.4681E-2</v>
+        <v>-2.01689E-2</v>
       </c>
       <c r="O4">
-        <v>7.4068899999999993E-2</v>
+        <v>7.6913200000000001E-2</v>
       </c>
       <c r="P4">
-        <v>0.14813899999999999</v>
+        <v>0.15154219999999999</v>
       </c>
       <c r="Q4">
-        <v>7.9184099999999993E-2</v>
+        <v>7.9776899999999998E-2</v>
       </c>
       <c r="R4">
-        <v>5.7914999999999998E-3</v>
+        <v>4.9397E-3</v>
       </c>
       <c r="S4">
-        <v>4.3156000000000002E-3</v>
+        <v>7.8470000000000005E-4</v>
       </c>
       <c r="T4">
-        <v>7.0089999999999996E-3</v>
+        <v>4.1939000000000004E-3</v>
       </c>
       <c r="U4">
-        <v>-0.10924200000000001</v>
+        <v>-0.110704</v>
       </c>
       <c r="V4">
-        <v>-9.6373500000000001E-2</v>
+        <v>-9.9208500000000005E-2</v>
       </c>
       <c r="W4">
-        <v>-0.1061272</v>
+        <v>-0.1135723</v>
       </c>
       <c r="X4">
-        <v>-0.10265249999999999</v>
+        <v>-0.1077231</v>
       </c>
       <c r="Y4">
-        <v>-1.43877E-2</v>
+        <v>-1.5681299999999999E-2</v>
       </c>
       <c r="Z4">
-        <v>-3.2142799999999999E-2</v>
+        <v>-3.56818E-2</v>
       </c>
       <c r="AA4">
-        <v>-0.13473760000000001</v>
+        <v>-0.14443220000000001</v>
       </c>
       <c r="AB4">
-        <v>-0.12691469999999999</v>
+        <v>-0.13511319999999999</v>
       </c>
       <c r="AC4">
-        <v>7.3300500000000005E-2</v>
+        <v>7.8125200000000006E-2</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.2">
@@ -1418,82 +1418,82 @@
         <v>32</v>
       </c>
       <c r="D5">
-        <v>2.6441300000000001E-2</v>
+        <v>3.2675299999999997E-2</v>
       </c>
       <c r="E5">
-        <v>0.1476905</v>
+        <v>0.16427</v>
       </c>
       <c r="F5">
-        <v>-0.28465980000000002</v>
+        <v>-0.29990410000000001</v>
       </c>
       <c r="G5" t="s">
         <v>29</v>
       </c>
       <c r="H5">
-        <v>-1.0491256</v>
+        <v>-1.1255729000000001</v>
       </c>
       <c r="I5">
-        <v>0.1217155</v>
+        <v>0.1333492</v>
       </c>
       <c r="J5">
-        <v>0.1514798</v>
+        <v>0.1653481</v>
       </c>
       <c r="K5">
-        <v>-3.16361E-2</v>
+        <v>-2.8441000000000001E-2</v>
       </c>
       <c r="L5">
-        <v>-8.6474999999999996E-2</v>
+        <v>-8.5712700000000003E-2</v>
       </c>
       <c r="M5">
-        <v>0.1016171</v>
+        <v>0.1114472</v>
       </c>
       <c r="N5">
-        <v>9.5584000000000002E-2</v>
+        <v>0.1076849</v>
       </c>
       <c r="O5">
-        <v>5.0727800000000003E-2</v>
+        <v>5.7562299999999997E-2</v>
       </c>
       <c r="P5">
-        <v>6.78647E-2</v>
+        <v>8.4873599999999993E-2</v>
       </c>
       <c r="Q5">
-        <v>9.2699999999999998E-4</v>
+        <v>-1.0544E-3</v>
       </c>
       <c r="R5">
-        <v>-7.4104199999999995E-2</v>
+        <v>-7.6425099999999996E-2</v>
       </c>
       <c r="S5">
-        <v>-5.6225600000000001E-2</v>
+        <v>-5.5075100000000002E-2</v>
       </c>
       <c r="T5">
-        <v>-7.3258299999999998E-2</v>
+        <v>-7.2293399999999994E-2</v>
       </c>
       <c r="U5">
-        <v>1.44972E-2</v>
+        <v>1.56477E-2</v>
       </c>
       <c r="V5">
-        <v>1.3952600000000001E-2</v>
+        <v>2.0500000000000001E-2</v>
       </c>
       <c r="W5">
-        <v>1.52248E-2</v>
+        <v>2.2694499999999999E-2</v>
       </c>
       <c r="X5">
-        <v>-2.9047999999999999E-3</v>
+        <v>-1.8259999999999999E-3</v>
       </c>
       <c r="Y5">
-        <v>-6.8396600000000002E-2</v>
+        <v>-7.0581699999999997E-2</v>
       </c>
       <c r="Z5">
-        <v>-6.2769000000000005E-2</v>
+        <v>-6.50057E-2</v>
       </c>
       <c r="AA5">
-        <v>-1.19077E-2</v>
+        <v>-4.0895000000000003E-3</v>
       </c>
       <c r="AB5">
-        <v>-2.5695800000000001E-2</v>
+        <v>-2.77536E-2</v>
       </c>
       <c r="AC5">
-        <v>-1.31614E-2</v>
+        <v>-9.7911999999999999E-3</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.2">
@@ -1504,82 +1504,82 @@
         <v>33</v>
       </c>
       <c r="D6">
-        <v>0.26716640000000003</v>
+        <v>0.28379939999999998</v>
       </c>
       <c r="E6">
-        <v>0.26529190000000002</v>
+        <v>0.28087400000000001</v>
       </c>
       <c r="F6">
-        <v>1.73572E-2</v>
+        <v>1.27776E-2</v>
       </c>
       <c r="G6">
-        <v>-0.41021190000000002</v>
+        <v>-0.45231369999999999</v>
       </c>
       <c r="H6" t="s">
         <v>29</v>
       </c>
       <c r="I6">
-        <v>0.22293080000000001</v>
+        <v>0.23675740000000001</v>
       </c>
       <c r="J6">
-        <v>0.17646719999999999</v>
+        <v>0.1829662</v>
       </c>
       <c r="K6">
-        <v>0.1402535</v>
+        <v>0.1487723</v>
       </c>
       <c r="L6">
-        <v>0.1482957</v>
+        <v>0.1529181</v>
       </c>
       <c r="M6">
-        <v>0.19797709999999999</v>
+        <v>0.2112436</v>
       </c>
       <c r="N6">
-        <v>0.16297780000000001</v>
+        <v>0.17645620000000001</v>
       </c>
       <c r="O6">
-        <v>0.1676937</v>
+        <v>0.17663860000000001</v>
       </c>
       <c r="P6">
-        <v>0.1961465</v>
+        <v>0.2060343</v>
       </c>
       <c r="Q6">
-        <v>0.1116613</v>
+        <v>0.1217077</v>
       </c>
       <c r="R6">
-        <v>4.1876299999999998E-2</v>
+        <v>4.3208700000000003E-2</v>
       </c>
       <c r="S6">
-        <v>4.3317300000000003E-2</v>
+        <v>4.5542300000000001E-2</v>
       </c>
       <c r="T6">
-        <v>3.7990500000000003E-2</v>
+        <v>3.9351700000000003E-2</v>
       </c>
       <c r="U6">
-        <v>8.4180599999999994E-2</v>
+        <v>9.4773700000000002E-2</v>
       </c>
       <c r="V6">
-        <v>7.73345E-2</v>
+        <v>9.1385599999999997E-2</v>
       </c>
       <c r="W6">
-        <v>6.5568399999999999E-2</v>
+        <v>7.46309E-2</v>
       </c>
       <c r="X6">
-        <v>6.5187999999999996E-2</v>
+        <v>7.4270000000000003E-2</v>
       </c>
       <c r="Y6">
-        <v>3.4354999999999997E-2</v>
+        <v>3.13762E-2</v>
       </c>
       <c r="Z6">
-        <v>3.3327299999999997E-2</v>
+        <v>3.5372599999999997E-2</v>
       </c>
       <c r="AA6">
-        <v>5.4957199999999998E-2</v>
+        <v>6.4063200000000001E-2</v>
       </c>
       <c r="AB6">
-        <v>5.7497300000000001E-2</v>
+        <v>6.8371000000000001E-2</v>
       </c>
       <c r="AC6">
-        <v>0.1993771</v>
+        <v>0.211868</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.2">
@@ -1593,82 +1593,82 @@
         <v>34</v>
       </c>
       <c r="D7">
-        <v>1.4811700000000001E-2</v>
+        <v>1.2057200000000001E-2</v>
       </c>
       <c r="E7">
-        <v>0.10690189999999999</v>
+        <v>0.1083322</v>
       </c>
       <c r="F7">
-        <v>-6.0661399999999997E-2</v>
+        <v>-7.1693699999999999E-2</v>
       </c>
       <c r="G7">
-        <v>5.3113500000000001E-2</v>
+        <v>5.5881599999999997E-2</v>
       </c>
       <c r="H7">
-        <v>7.7620099999999997E-2</v>
+        <v>7.9830499999999999E-2</v>
       </c>
       <c r="I7" t="s">
         <v>29</v>
       </c>
       <c r="J7">
-        <v>-1.3299363</v>
+        <v>-1.4029564000000001</v>
       </c>
       <c r="K7">
-        <v>-5.6686300000000002E-2</v>
+        <v>-5.9030199999999998E-2</v>
       </c>
       <c r="L7">
-        <v>-3.9534699999999999E-2</v>
+        <v>-3.8996500000000003E-2</v>
       </c>
       <c r="M7">
-        <v>3.2316299999999999E-2</v>
+        <v>1.04402E-2</v>
       </c>
       <c r="N7">
-        <v>-3.1275999999999999E-3</v>
+        <v>-1.20041E-2</v>
       </c>
       <c r="O7">
-        <v>0.1616563</v>
+        <v>0.15168509999999999</v>
       </c>
       <c r="P7">
-        <v>9.93251E-2</v>
+        <v>9.8213400000000006E-2</v>
       </c>
       <c r="Q7">
-        <v>-6.15297E-2</v>
+        <v>-7.1540199999999998E-2</v>
       </c>
       <c r="R7">
-        <v>-8.7665300000000002E-2</v>
+        <v>-9.3714900000000004E-2</v>
       </c>
       <c r="S7">
-        <v>-9.8118300000000006E-2</v>
+        <v>-0.1067253</v>
       </c>
       <c r="T7">
-        <v>-4.2787600000000002E-2</v>
+        <v>-4.57563E-2</v>
       </c>
       <c r="U7">
-        <v>-3.8437499999999999E-2</v>
+        <v>-4.2761800000000003E-2</v>
       </c>
       <c r="V7">
-        <v>-7.03294E-2</v>
+        <v>-7.7829800000000005E-2</v>
       </c>
       <c r="W7">
-        <v>-6.33412E-2</v>
+        <v>-7.19915E-2</v>
       </c>
       <c r="X7">
-        <v>-5.5204999999999997E-2</v>
+        <v>-6.2837000000000004E-2</v>
       </c>
       <c r="Y7">
-        <v>1.2319099999999999E-2</v>
+        <v>1.7634199999999999E-2</v>
       </c>
       <c r="Z7">
-        <v>4.2739199999999998E-2</v>
+        <v>4.5198599999999998E-2</v>
       </c>
       <c r="AA7">
-        <v>2.9582899999999999E-2</v>
+        <v>3.1140000000000001E-2</v>
       </c>
       <c r="AB7">
-        <v>-4.5245899999999999E-2</v>
+        <v>-5.0265600000000001E-2</v>
       </c>
       <c r="AC7">
-        <v>-0.12726460000000001</v>
+        <v>-0.13344800000000001</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.2">
@@ -1682,82 +1682,82 @@
         <v>35</v>
       </c>
       <c r="D8">
-        <v>0.20730299999999999</v>
+        <v>0.21530750000000001</v>
       </c>
       <c r="E8">
-        <v>0.12419139999999999</v>
+        <v>0.1214596</v>
       </c>
       <c r="F8">
-        <v>2.7719199999999999E-2</v>
+        <v>2.8069E-2</v>
       </c>
       <c r="G8">
-        <v>0.12828200000000001</v>
+        <v>0.123265</v>
       </c>
       <c r="H8">
-        <v>-8.0406999999999996E-3</v>
+        <v>-2.3395900000000001E-2</v>
       </c>
       <c r="I8">
-        <v>-1.1108297</v>
+        <v>-1.1535481999999999</v>
       </c>
       <c r="J8" t="s">
         <v>29</v>
       </c>
       <c r="K8">
-        <v>8.8675100000000007E-2</v>
+        <v>9.3407400000000002E-2</v>
       </c>
       <c r="L8">
-        <v>-9.136E-3</v>
+        <v>-1.50105E-2</v>
       </c>
       <c r="M8">
-        <v>0.13515720000000001</v>
+        <v>0.14948790000000001</v>
       </c>
       <c r="N8">
-        <v>0.30198710000000001</v>
+        <v>0.31198379999999998</v>
       </c>
       <c r="O8">
-        <v>0.17088439999999999</v>
+        <v>0.17746300000000001</v>
       </c>
       <c r="P8">
-        <v>5.1257900000000002E-2</v>
+        <v>5.60545E-2</v>
       </c>
       <c r="Q8">
-        <v>0.1491722</v>
+        <v>0.1616215</v>
       </c>
       <c r="R8">
-        <v>-3.3179100000000003E-2</v>
+        <v>-4.1225400000000002E-2</v>
       </c>
       <c r="S8">
-        <v>-3.1337000000000001E-3</v>
+        <v>-6.1641999999999999E-3</v>
       </c>
       <c r="T8">
-        <v>-5.4692200000000003E-2</v>
+        <v>-6.5239199999999997E-2</v>
       </c>
       <c r="U8">
-        <v>7.5451099999999993E-2</v>
+        <v>7.1354000000000001E-2</v>
       </c>
       <c r="V8">
-        <v>5.78018E-2</v>
+        <v>6.0580700000000001E-2</v>
       </c>
       <c r="W8">
-        <v>-3.3535299999999997E-2</v>
+        <v>-3.1049199999999999E-2</v>
       </c>
       <c r="X8">
-        <v>-1.5485199999999999E-2</v>
+        <v>-1.25366E-2</v>
       </c>
       <c r="Y8">
-        <v>2.4324399999999999E-2</v>
+        <v>2.1552999999999999E-2</v>
       </c>
       <c r="Z8">
-        <v>4.8767999999999999E-2</v>
+        <v>4.5180900000000003E-2</v>
       </c>
       <c r="AA8">
-        <v>9.6226500000000006E-2</v>
+        <v>9.1601500000000002E-2</v>
       </c>
       <c r="AB8">
-        <v>7.6419000000000001E-3</v>
+        <v>3.3565999999999999E-3</v>
       </c>
       <c r="AC8">
-        <v>2.0075900000000001E-2</v>
+        <v>1.7342699999999999E-2</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.2">
@@ -1768,82 +1768,82 @@
         <v>36</v>
       </c>
       <c r="D9">
-        <v>4.1466999999999997E-2</v>
+        <v>4.45114E-2</v>
       </c>
       <c r="E9">
-        <v>5.9743200000000003E-2</v>
+        <v>6.0080799999999997E-2</v>
       </c>
       <c r="F9">
-        <v>1.1712999999999999E-2</v>
+        <v>1.17728E-2</v>
       </c>
       <c r="G9">
-        <v>1.43356E-2</v>
+        <v>1.7608700000000001E-2</v>
       </c>
       <c r="H9">
-        <v>-3.4668499999999998E-2</v>
+        <v>-3.2796499999999999E-2</v>
       </c>
       <c r="I9">
-        <v>-2.9364100000000001E-2</v>
+        <v>-2.5989700000000001E-2</v>
       </c>
       <c r="J9">
-        <v>-2.27382E-2</v>
+        <v>-1.4501E-2</v>
       </c>
       <c r="K9" t="s">
         <v>29</v>
       </c>
       <c r="L9">
-        <v>-0.62522080000000002</v>
+        <v>-0.66993559999999996</v>
       </c>
       <c r="M9">
-        <v>4.4183100000000003E-2</v>
+        <v>5.0610299999999997E-2</v>
       </c>
       <c r="N9">
-        <v>5.3368800000000001E-2</v>
+        <v>5.8596299999999997E-2</v>
       </c>
       <c r="O9">
-        <v>9.2193700000000003E-2</v>
+        <v>0.101354</v>
       </c>
       <c r="P9">
-        <v>6.2786499999999995E-2</v>
+        <v>6.3603499999999993E-2</v>
       </c>
       <c r="Q9">
-        <v>-2.3481200000000001E-2</v>
+        <v>-2.1807400000000001E-2</v>
       </c>
       <c r="R9">
-        <v>1.951E-3</v>
+        <v>1.6402000000000001E-3</v>
       </c>
       <c r="S9">
-        <v>2.0278999999999998E-2</v>
+        <v>2.1834599999999999E-2</v>
       </c>
       <c r="T9">
-        <v>-6.0717999999999996E-3</v>
+        <v>-9.4511999999999999E-3</v>
       </c>
       <c r="U9">
-        <v>-0.10236290000000001</v>
+        <v>-0.1115527</v>
       </c>
       <c r="V9">
-        <v>1.4085200000000001E-2</v>
+        <v>1.7563100000000002E-2</v>
       </c>
       <c r="W9">
-        <v>4.6452199999999999E-2</v>
+        <v>4.8421699999999998E-2</v>
       </c>
       <c r="X9">
-        <v>1.9219199999999999E-2</v>
+        <v>2.1411900000000001E-2</v>
       </c>
       <c r="Y9">
-        <v>-5.2098999999999999E-2</v>
+        <v>-6.0673499999999998E-2</v>
       </c>
       <c r="Z9">
-        <v>-5.3325499999999998E-2</v>
+        <v>-6.5807199999999996E-2</v>
       </c>
       <c r="AA9">
-        <v>-8.5491499999999998E-2</v>
+        <v>-8.9249300000000004E-2</v>
       </c>
       <c r="AB9">
-        <v>-0.13310169999999999</v>
+        <v>-0.13686139999999999</v>
       </c>
       <c r="AC9">
-        <v>-6.8027599999999994E-2</v>
+        <v>-6.0967100000000003E-2</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
@@ -1854,82 +1854,82 @@
         <v>37</v>
       </c>
       <c r="D10">
-        <v>0.2324543</v>
+        <v>0.25192399999999998</v>
       </c>
       <c r="E10">
-        <v>0.2247941</v>
+        <v>0.24093129999999999</v>
       </c>
       <c r="F10">
-        <v>0.26174330000000001</v>
+        <v>0.28114800000000001</v>
       </c>
       <c r="G10">
-        <v>0.16943169999999999</v>
+        <v>0.17825199999999999</v>
       </c>
       <c r="H10">
-        <v>0.18950819999999999</v>
+        <v>0.2038741</v>
       </c>
       <c r="I10">
-        <v>0.21200949999999999</v>
+        <v>0.2323211</v>
       </c>
       <c r="J10">
-        <v>0.14291970000000001</v>
+        <v>0.15141769999999999</v>
       </c>
       <c r="K10">
-        <v>-8.6766899999999994E-2</v>
+        <v>-9.2431399999999997E-2</v>
       </c>
       <c r="L10" t="s">
         <v>29</v>
       </c>
       <c r="M10">
-        <v>0.1241478</v>
+        <v>0.13510449999999999</v>
       </c>
       <c r="N10">
-        <v>0.1457743</v>
+        <v>0.15370159999999999</v>
       </c>
       <c r="O10">
-        <v>9.4306899999999999E-2</v>
+        <v>0.10074139999999999</v>
       </c>
       <c r="P10">
-        <v>0.18100640000000001</v>
+        <v>0.2008037</v>
       </c>
       <c r="Q10">
-        <v>-2.6111599999999999E-2</v>
+        <v>-3.01306E-2</v>
       </c>
       <c r="R10">
-        <v>8.4522E-3</v>
+        <v>7.7950000000000003E-4</v>
       </c>
       <c r="S10">
-        <v>2.5245E-2</v>
+        <v>1.53743E-2</v>
       </c>
       <c r="T10">
-        <v>-1.2464100000000001E-2</v>
+        <v>-2.1564699999999999E-2</v>
       </c>
       <c r="U10">
-        <v>-9.9446999999999994E-2</v>
+        <v>-0.1054918</v>
       </c>
       <c r="V10">
-        <v>-3.95152E-2</v>
+        <v>-4.2941199999999999E-2</v>
       </c>
       <c r="W10">
-        <v>-6.3096799999999995E-2</v>
+        <v>-6.9263599999999995E-2</v>
       </c>
       <c r="X10">
-        <v>-7.7463400000000002E-2</v>
+        <v>-8.3567100000000005E-2</v>
       </c>
       <c r="Y10">
-        <v>-4.8519600000000003E-2</v>
+        <v>-5.32807E-2</v>
       </c>
       <c r="Z10">
-        <v>-4.8456300000000001E-2</v>
+        <v>-5.2096200000000002E-2</v>
       </c>
       <c r="AA10">
-        <v>-8.6644499999999999E-2</v>
+        <v>-9.8362599999999994E-2</v>
       </c>
       <c r="AB10">
-        <v>-0.1103394</v>
+        <v>-0.1239021</v>
       </c>
       <c r="AC10">
-        <v>0.1000077</v>
+        <v>0.1020995</v>
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.2">
@@ -1943,82 +1943,82 @@
         <v>38</v>
       </c>
       <c r="D11">
-        <v>3.3712899999999997E-2</v>
+        <v>3.2856400000000001E-2</v>
       </c>
       <c r="E11">
-        <v>9.0787099999999996E-2</v>
+        <v>9.2385700000000001E-2</v>
       </c>
       <c r="F11">
-        <v>8.5246100000000005E-2</v>
+        <v>8.1215099999999998E-2</v>
       </c>
       <c r="G11">
-        <v>8.1556199999999995E-2</v>
+        <v>8.3129599999999998E-2</v>
       </c>
       <c r="H11">
-        <v>0.1087549</v>
+        <v>0.11054700000000001</v>
       </c>
       <c r="I11">
-        <v>-6.5693699999999994E-2</v>
+        <v>-7.8040899999999996E-2</v>
       </c>
       <c r="J11">
-        <v>-4.5766599999999998E-2</v>
+        <v>-5.3201900000000003E-2</v>
       </c>
       <c r="K11">
-        <v>7.7265399999999998E-2</v>
+        <v>8.2696599999999995E-2</v>
       </c>
       <c r="L11">
-        <v>-4.5699400000000001E-2</v>
+        <v>-4.27745E-2</v>
       </c>
       <c r="M11" t="s">
         <v>29</v>
       </c>
       <c r="N11">
-        <v>-0.13897689999999999</v>
+        <v>-0.14342240000000001</v>
       </c>
       <c r="O11">
-        <v>-0.26963920000000002</v>
+        <v>-0.28022659999999999</v>
       </c>
       <c r="P11">
-        <v>-7.5619500000000006E-2</v>
+        <v>-7.0421399999999995E-2</v>
       </c>
       <c r="Q11">
-        <v>-0.16862959999999999</v>
+        <v>-0.17400570000000001</v>
       </c>
       <c r="R11">
-        <v>-5.2622599999999999E-2</v>
+        <v>-4.0385400000000002E-2</v>
       </c>
       <c r="S11">
-        <v>-3.3572400000000002E-2</v>
+        <v>-2.0927500000000002E-2</v>
       </c>
       <c r="T11">
-        <v>-4.1333700000000001E-2</v>
+        <v>-3.1651899999999997E-2</v>
       </c>
       <c r="U11">
-        <v>-0.23320579999999999</v>
+        <v>-0.2518087</v>
       </c>
       <c r="V11">
-        <v>-4.9454400000000003E-2</v>
+        <v>-5.7203900000000002E-2</v>
       </c>
       <c r="W11">
-        <v>-0.1286323</v>
+        <v>-0.1381231</v>
       </c>
       <c r="X11">
-        <v>-6.52866E-2</v>
+        <v>-7.0716600000000004E-2</v>
       </c>
       <c r="Y11">
-        <v>-0.116937</v>
+        <v>-0.11581660000000001</v>
       </c>
       <c r="Z11">
-        <v>-0.1040502</v>
+        <v>-0.10645309999999999</v>
       </c>
       <c r="AA11">
-        <v>-0.1781596</v>
+        <v>-0.189494</v>
       </c>
       <c r="AB11">
-        <v>-0.13196820000000001</v>
+        <v>-0.1468024</v>
       </c>
       <c r="AC11">
-        <v>-3.2319899999999999E-2</v>
+        <v>-3.5550699999999998E-2</v>
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
@@ -2032,82 +2032,82 @@
         <v>39</v>
       </c>
       <c r="D12">
-        <v>-3.4609800000000003E-2</v>
+        <v>-4.3525000000000001E-2</v>
       </c>
       <c r="E12">
-        <v>1.17821E-2</v>
+        <v>-2.062E-4</v>
       </c>
       <c r="F12">
-        <v>-7.6312400000000002E-2</v>
+        <v>-8.17166E-2</v>
       </c>
       <c r="G12">
-        <v>-4.1258000000000003E-2</v>
+        <v>-4.35573E-2</v>
       </c>
       <c r="H12">
-        <v>2.7786100000000001E-2</v>
+        <v>3.3534300000000003E-2</v>
       </c>
       <c r="I12">
-        <v>-9.9673000000000001E-3</v>
+        <v>-6.7901999999999997E-3</v>
       </c>
       <c r="J12">
-        <v>9.0077000000000004E-2</v>
+        <v>9.7019499999999995E-2</v>
       </c>
       <c r="K12">
-        <v>-5.1612400000000003E-2</v>
+        <v>-5.0801399999999997E-2</v>
       </c>
       <c r="L12">
-        <v>-3.1863700000000002E-2</v>
+        <v>-3.1980399999999999E-2</v>
       </c>
       <c r="M12">
-        <v>-0.20005419999999999</v>
+        <v>-0.1969052</v>
       </c>
       <c r="N12" t="s">
         <v>29</v>
       </c>
       <c r="O12">
-        <v>-0.50705880000000003</v>
+        <v>-0.52103259999999996</v>
       </c>
       <c r="P12">
-        <v>-6.3783800000000002E-2</v>
+        <v>-6.5257499999999996E-2</v>
       </c>
       <c r="Q12">
-        <v>7.528E-3</v>
+        <v>1.0814300000000001E-2</v>
       </c>
       <c r="R12">
-        <v>-1.96705E-2</v>
+        <v>-2.22499E-2</v>
       </c>
       <c r="S12">
-        <v>-3.8790999999999999E-2</v>
+        <v>-4.5852400000000001E-2</v>
       </c>
       <c r="T12">
-        <v>-6.9789900000000002E-2</v>
+        <v>-7.7755900000000003E-2</v>
       </c>
       <c r="U12">
-        <v>7.3728100000000005E-2</v>
+        <v>7.9123799999999994E-2</v>
       </c>
       <c r="V12">
-        <v>2.3246900000000001E-2</v>
+        <v>2.5450400000000001E-2</v>
       </c>
       <c r="W12">
-        <v>5.2749900000000002E-2</v>
+        <v>5.6384299999999998E-2</v>
       </c>
       <c r="X12">
-        <v>5.5327300000000003E-2</v>
+        <v>6.1252399999999999E-2</v>
       </c>
       <c r="Y12">
-        <v>1.7473200000000001E-2</v>
+        <v>1.43476E-2</v>
       </c>
       <c r="Z12">
-        <v>2.1608999999999999E-3</v>
+        <v>9.5989999999999997E-4</v>
       </c>
       <c r="AA12">
-        <v>-1.2318900000000001E-2</v>
+        <v>-4.6484999999999999E-3</v>
       </c>
       <c r="AB12">
-        <v>5.4375E-2</v>
+        <v>6.17131E-2</v>
       </c>
       <c r="AC12">
-        <v>7.4020600000000006E-2</v>
+        <v>7.8049599999999997E-2</v>
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.2">
@@ -2121,82 +2121,82 @@
         <v>40</v>
       </c>
       <c r="D13">
-        <v>0.31640990000000002</v>
+        <v>0.3308932</v>
       </c>
       <c r="E13">
-        <v>0.2045498</v>
+        <v>0.21274019999999999</v>
       </c>
       <c r="F13">
-        <v>0.30621730000000003</v>
+        <v>0.32165850000000001</v>
       </c>
       <c r="G13">
-        <v>0.19294459999999999</v>
+        <v>0.20295440000000001</v>
       </c>
       <c r="H13">
-        <v>0.23878350000000001</v>
+        <v>0.24610489999999999</v>
       </c>
       <c r="I13">
-        <v>0.42177140000000002</v>
+        <v>0.43989080000000003</v>
       </c>
       <c r="J13">
-        <v>0.38585249999999999</v>
+        <v>0.39965119999999998</v>
       </c>
       <c r="K13">
-        <v>0.1707359</v>
+        <v>0.17753930000000001</v>
       </c>
       <c r="L13">
-        <v>0.18022369999999999</v>
+        <v>0.18358469999999999</v>
       </c>
       <c r="M13">
-        <v>0.204933</v>
+        <v>0.21674579999999999</v>
       </c>
       <c r="N13">
-        <v>4.14606E-2</v>
+        <v>4.8354000000000001E-2</v>
       </c>
       <c r="O13" t="s">
         <v>29</v>
       </c>
       <c r="P13">
-        <v>2.46368E-2</v>
+        <v>2.67348E-2</v>
       </c>
       <c r="Q13">
-        <v>2.2785799999999998E-2</v>
+        <v>9.3805999999999994E-3</v>
       </c>
       <c r="R13">
-        <v>5.5050799999999997E-2</v>
+        <v>5.2357099999999997E-2</v>
       </c>
       <c r="S13">
-        <v>6.0898000000000002E-3</v>
+        <v>3.3974999999999999E-3</v>
       </c>
       <c r="T13">
-        <v>4.9930200000000001E-2</v>
+        <v>5.2652999999999998E-2</v>
       </c>
       <c r="U13">
-        <v>0.12072479999999999</v>
+        <v>0.1281775</v>
       </c>
       <c r="V13">
-        <v>0.3758843</v>
+        <v>0.39963510000000002</v>
       </c>
       <c r="W13">
-        <v>0.36617749999999999</v>
+        <v>0.38139699999999999</v>
       </c>
       <c r="X13">
-        <v>0.3686876</v>
+        <v>0.38569730000000002</v>
       </c>
       <c r="Y13">
-        <v>0.15366779999999999</v>
+        <v>0.1638096</v>
       </c>
       <c r="Z13">
-        <v>0.12691820000000001</v>
+        <v>0.1337468</v>
       </c>
       <c r="AA13">
-        <v>0.16036239999999999</v>
+        <v>0.16194629999999999</v>
       </c>
       <c r="AB13">
-        <v>0.1198282</v>
+        <v>0.12223150000000001</v>
       </c>
       <c r="AC13">
-        <v>0.30556339999999999</v>
+        <v>0.32359369999999998</v>
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.2">
@@ -2210,82 +2210,82 @@
         <v>41</v>
       </c>
       <c r="D14">
-        <v>7.2051900000000002E-2</v>
+        <v>6.2869800000000003E-2</v>
       </c>
       <c r="E14">
-        <v>6.0989000000000002E-2</v>
+        <v>6.0452100000000002E-2</v>
       </c>
       <c r="F14">
-        <v>0.22664029999999999</v>
+        <v>0.23163790000000001</v>
       </c>
       <c r="G14">
-        <v>0.1145823</v>
+        <v>0.1112255</v>
       </c>
       <c r="H14">
-        <v>9.0446299999999993E-2</v>
+        <v>8.6558599999999999E-2</v>
       </c>
       <c r="I14">
-        <v>0.23647940000000001</v>
+        <v>0.23708679999999999</v>
       </c>
       <c r="J14">
-        <v>0.1279004</v>
+        <v>0.125637</v>
       </c>
       <c r="K14">
-        <v>0.1667526</v>
+        <v>0.1651223</v>
       </c>
       <c r="L14">
-        <v>0.14796519999999999</v>
+        <v>0.15063570000000001</v>
       </c>
       <c r="M14">
-        <v>-2.12356E-2</v>
+        <v>-2.07484E-2</v>
       </c>
       <c r="N14">
-        <v>-7.0569800000000002E-2</v>
+        <v>-7.8051400000000007E-2</v>
       </c>
       <c r="O14">
-        <v>-0.27471060000000003</v>
+        <v>-0.29412919999999998</v>
       </c>
       <c r="P14" t="s">
         <v>29</v>
       </c>
       <c r="Q14">
-        <v>-0.28664899999999999</v>
+        <v>-0.29800759999999998</v>
       </c>
       <c r="R14">
-        <v>-2.70502E-2</v>
+        <v>-3.99377E-2</v>
       </c>
       <c r="S14">
-        <v>2.8595800000000001E-2</v>
+        <v>1.9799799999999999E-2</v>
       </c>
       <c r="T14">
-        <v>1.37045E-2</v>
+        <v>8.7957E-3</v>
       </c>
       <c r="U14">
-        <v>-8.6721999999999994E-2</v>
+        <v>-9.60038E-2</v>
       </c>
       <c r="V14">
-        <v>4.8497999999999996E-3</v>
+        <v>-7.7464999999999999E-3</v>
       </c>
       <c r="W14">
-        <v>-1.50131E-2</v>
+        <v>-1.9262700000000001E-2</v>
       </c>
       <c r="X14">
-        <v>-6.0299100000000001E-2</v>
+        <v>-7.2726100000000002E-2</v>
       </c>
       <c r="Y14">
-        <v>1.9938899999999999E-2</v>
+        <v>1.6822500000000001E-2</v>
       </c>
       <c r="Z14">
-        <v>-9.8919999999999998E-4</v>
+        <v>-6.3350000000000004E-3</v>
       </c>
       <c r="AA14">
-        <v>-0.13093050000000001</v>
+        <v>-0.14132620000000001</v>
       </c>
       <c r="AB14">
-        <v>-0.10487150000000001</v>
+        <v>-0.116697</v>
       </c>
       <c r="AC14">
-        <v>-1.09062E-2</v>
+        <v>-2.9398899999999999E-2</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.2">
@@ -2299,82 +2299,82 @@
         <v>42</v>
       </c>
       <c r="D15">
-        <v>-5.2760000000000001E-2</v>
+        <v>-6.4491599999999996E-2</v>
       </c>
       <c r="E15">
-        <v>-2.76893E-2</v>
+        <v>-3.2345199999999998E-2</v>
       </c>
       <c r="F15">
-        <v>2.5383599999999999E-2</v>
+        <v>1.9484100000000001E-2</v>
       </c>
       <c r="G15">
-        <v>4.5247099999999998E-2</v>
+        <v>4.02473E-2</v>
       </c>
       <c r="H15">
-        <v>3.9114400000000001E-2</v>
+        <v>3.3155999999999998E-2</v>
       </c>
       <c r="I15">
-        <v>-0.1014592</v>
+        <v>-0.10879809999999999</v>
       </c>
       <c r="J15">
-        <v>-5.0130599999999997E-2</v>
+        <v>-6.13987E-2</v>
       </c>
       <c r="K15">
-        <v>-0.121166</v>
+        <v>-0.1326821</v>
       </c>
       <c r="L15">
-        <v>-0.15059549999999999</v>
+        <v>-0.16028390000000001</v>
       </c>
       <c r="M15">
-        <v>3.3984199999999999E-2</v>
+        <v>2.9916499999999999E-2</v>
       </c>
       <c r="N15">
-        <v>-9.0981300000000001E-2</v>
+        <v>-0.1019786</v>
       </c>
       <c r="O15">
-        <v>1.2711999999999999E-2</v>
+        <v>9.1902000000000008E-3</v>
       </c>
       <c r="P15">
-        <v>-0.124211</v>
+        <v>-0.13200110000000001</v>
       </c>
       <c r="Q15" t="s">
         <v>29</v>
       </c>
       <c r="R15">
-        <v>-0.11251129999999999</v>
+        <v>-0.12886980000000001</v>
       </c>
       <c r="S15">
-        <v>-3.3666799999999997E-2</v>
+        <v>-4.6618399999999997E-2</v>
       </c>
       <c r="T15">
-        <v>-8.5009699999999994E-2</v>
+        <v>-9.7578200000000004E-2</v>
       </c>
       <c r="U15">
-        <v>-1.1435799999999999E-2</v>
+        <v>-1.44831E-2</v>
       </c>
       <c r="V15">
-        <v>-6.7393599999999998E-2</v>
+        <v>-7.7899499999999997E-2</v>
       </c>
       <c r="W15">
-        <v>-5.4499100000000002E-2</v>
+        <v>-6.6278400000000001E-2</v>
       </c>
       <c r="X15">
-        <v>-9.8131200000000002E-2</v>
+        <v>-0.1104908</v>
       </c>
       <c r="Y15">
-        <v>-2.7129500000000001E-2</v>
+        <v>-2.9712100000000002E-2</v>
       </c>
       <c r="Z15">
-        <v>-2.4785100000000001E-2</v>
+        <v>-2.8005200000000001E-2</v>
       </c>
       <c r="AA15">
-        <v>1.9658200000000001E-2</v>
+        <v>1.6062400000000001E-2</v>
       </c>
       <c r="AB15">
-        <v>-1.3724800000000001E-2</v>
+        <v>-1.7358599999999998E-2</v>
       </c>
       <c r="AC15">
-        <v>-3.9777100000000003E-2</v>
+        <v>-3.8909800000000001E-2</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.2">
@@ -2388,82 +2388,82 @@
         <v>43</v>
       </c>
       <c r="D16">
-        <v>7.8521300000000002E-2</v>
+        <v>8.8963200000000006E-2</v>
       </c>
       <c r="E16">
-        <v>0.1651514</v>
+        <v>0.1681994</v>
       </c>
       <c r="F16">
-        <v>0.1185721</v>
+        <v>0.1315885</v>
       </c>
       <c r="G16">
-        <v>9.1218300000000002E-2</v>
+        <v>9.5569799999999996E-2</v>
       </c>
       <c r="H16">
-        <v>8.6317699999999997E-2</v>
+        <v>8.9054700000000001E-2</v>
       </c>
       <c r="I16">
-        <v>-5.5070300000000003E-2</v>
+        <v>-7.6930799999999994E-2</v>
       </c>
       <c r="J16">
-        <v>-2.07414E-2</v>
+        <v>-3.7816799999999998E-2</v>
       </c>
       <c r="K16">
-        <v>0.1021869</v>
+        <v>0.10028769999999999</v>
       </c>
       <c r="L16">
-        <v>0.1117659</v>
+        <v>0.1062732</v>
       </c>
       <c r="M16">
-        <v>-3.0325499999999998E-2</v>
+        <v>-4.0610599999999997E-2</v>
       </c>
       <c r="N16">
-        <v>-1.5255299999999999E-2</v>
+        <v>-3.32953E-2</v>
       </c>
       <c r="O16">
-        <v>-1.7559700000000001E-2</v>
+        <v>-3.1702899999999999E-2</v>
       </c>
       <c r="P16">
-        <v>-0.10075729999999999</v>
+        <v>-0.13410730000000001</v>
       </c>
       <c r="Q16">
-        <v>-4.5037800000000003E-2</v>
+        <v>-5.7487900000000001E-2</v>
       </c>
       <c r="R16" t="s">
         <v>29</v>
       </c>
       <c r="S16">
-        <v>-0.1860146</v>
+        <v>-0.23831730000000001</v>
       </c>
       <c r="T16">
-        <v>-0.20358219999999999</v>
+        <v>-0.25328410000000001</v>
       </c>
       <c r="U16">
-        <v>-2.20488E-2</v>
+        <v>-4.8110699999999999E-2</v>
       </c>
       <c r="V16">
-        <v>7.6220000000000003E-3</v>
+        <v>-1.4191499999999999E-2</v>
       </c>
       <c r="W16">
-        <v>-1.4999500000000001E-2</v>
-      </c>
-      <c r="X16" s="1">
-        <v>8.1500000000000002E-5</v>
+        <v>-3.9801299999999998E-2</v>
+      </c>
+      <c r="X16">
+        <v>-2.13355E-2</v>
       </c>
       <c r="Y16">
-        <v>4.85224E-2</v>
+        <v>4.2170199999999998E-2</v>
       </c>
       <c r="Z16">
-        <v>2.91696E-2</v>
+        <v>1.6858499999999998E-2</v>
       </c>
       <c r="AA16">
-        <v>6.3666899999999998E-2</v>
+        <v>4.7596800000000002E-2</v>
       </c>
       <c r="AB16">
-        <v>-9.4879999999999999E-3</v>
+        <v>-2.3683900000000001E-2</v>
       </c>
       <c r="AC16">
-        <v>5.2491900000000001E-2</v>
+        <v>5.4049899999999998E-2</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.2">
@@ -2476,83 +2476,83 @@
       <c r="C17" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="1">
-        <v>-6.0300000000000002E-5</v>
+      <c r="D17">
+        <v>-5.3978000000000003E-3</v>
       </c>
       <c r="E17">
-        <v>6.2105500000000001E-2</v>
+        <v>6.3399999999999998E-2</v>
       </c>
       <c r="F17">
-        <v>2.64969E-2</v>
+        <v>2.2192900000000002E-2</v>
       </c>
       <c r="G17">
-        <v>4.26092E-2</v>
+        <v>4.3947E-2</v>
       </c>
       <c r="H17">
-        <v>4.6962499999999997E-2</v>
+        <v>4.5028400000000003E-2</v>
       </c>
       <c r="I17">
-        <v>-5.0901999999999996E-3</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="J17">
-        <v>-2.2780999999999999E-3</v>
+        <v>1.24633E-2</v>
       </c>
       <c r="K17">
-        <v>0.1041711</v>
+        <v>0.1029283</v>
       </c>
       <c r="L17">
-        <v>0.10218000000000001</v>
+        <v>0.10604239999999999</v>
       </c>
       <c r="M17">
-        <v>7.2338899999999998E-2</v>
+        <v>7.7170500000000003E-2</v>
       </c>
       <c r="N17">
-        <v>3.5819499999999997E-2</v>
+        <v>4.0030099999999999E-2</v>
       </c>
       <c r="O17">
-        <v>1.44701E-2</v>
+        <v>2.1163499999999998E-2</v>
       </c>
       <c r="P17">
-        <v>2.0962100000000001E-2</v>
+        <v>1.8921400000000001E-2</v>
       </c>
       <c r="Q17">
-        <v>-1.5034799999999999E-2</v>
+        <v>-2.1454399999999998E-2</v>
       </c>
       <c r="R17">
-        <v>-0.3169613</v>
+        <v>-0.33267839999999999</v>
       </c>
       <c r="S17" t="s">
         <v>29</v>
       </c>
       <c r="T17">
-        <v>-0.2751981</v>
+        <v>-0.29663430000000002</v>
       </c>
       <c r="U17">
-        <v>-7.3918899999999996E-2</v>
+        <v>-7.0441100000000006E-2</v>
       </c>
       <c r="V17">
-        <v>-1.61549E-2</v>
+        <v>-1.1042E-2</v>
       </c>
       <c r="W17">
-        <v>-1.17064E-2</v>
+        <v>-7.3223999999999997E-3</v>
       </c>
       <c r="X17">
-        <v>-2.3695600000000001E-2</v>
+        <v>-1.6734700000000002E-2</v>
       </c>
       <c r="Y17">
-        <v>-2.26938E-2</v>
+        <v>-2.5695900000000001E-2</v>
       </c>
       <c r="Z17">
-        <v>-3.4786600000000001E-2</v>
+        <v>-3.6612899999999997E-2</v>
       </c>
       <c r="AA17">
-        <v>1.4522800000000001E-2</v>
+        <v>1.8096000000000001E-2</v>
       </c>
       <c r="AB17">
-        <v>-5.95428E-2</v>
+        <v>-6.1266000000000001E-2</v>
       </c>
       <c r="AC17">
-        <v>2.76952E-2</v>
+        <v>2.9101599999999998E-2</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.2">
@@ -2566,82 +2566,82 @@
         <v>45</v>
       </c>
       <c r="D18">
-        <v>0.10159079999999999</v>
+        <v>0.1085335</v>
       </c>
       <c r="E18">
-        <v>0.17507320000000001</v>
+        <v>0.1846564</v>
       </c>
       <c r="F18">
-        <v>0.11700530000000001</v>
+        <v>0.1285144</v>
       </c>
       <c r="G18">
-        <v>9.2856499999999995E-2</v>
+        <v>0.1033599</v>
       </c>
       <c r="H18">
-        <v>8.9212799999999995E-2</v>
+        <v>9.9942199999999995E-2</v>
       </c>
       <c r="I18">
-        <v>-8.9449500000000001E-2</v>
+        <v>-9.2247700000000002E-2</v>
       </c>
       <c r="J18">
-        <v>-6.8545200000000001E-2</v>
+        <v>-7.6094899999999993E-2</v>
       </c>
       <c r="K18">
-        <v>7.6233400000000007E-2</v>
+        <v>8.7414500000000006E-2</v>
       </c>
       <c r="L18">
-        <v>7.1546799999999994E-2</v>
+        <v>8.1158999999999995E-2</v>
       </c>
       <c r="M18">
-        <v>2.8085499999999999E-2</v>
+        <v>2.6596600000000001E-2</v>
       </c>
       <c r="N18">
-        <v>-4.3628E-3</v>
+        <v>-2.9979E-3</v>
       </c>
       <c r="O18">
-        <v>3.9197000000000003E-2</v>
+        <v>4.2082300000000003E-2</v>
       </c>
       <c r="P18">
-        <v>-8.4336499999999995E-2</v>
+        <v>-8.7396600000000005E-2</v>
       </c>
       <c r="Q18">
-        <v>7.7230099999999996E-2</v>
+        <v>8.0716999999999997E-2</v>
       </c>
       <c r="R18">
-        <v>-0.24924830000000001</v>
+        <v>-0.25527430000000001</v>
       </c>
       <c r="S18">
-        <v>-0.18842790000000001</v>
+        <v>-0.1938532</v>
       </c>
       <c r="T18" t="s">
         <v>29</v>
       </c>
       <c r="U18">
-        <v>-3.5354700000000003E-2</v>
+        <v>-3.2303600000000002E-2</v>
       </c>
       <c r="V18">
-        <v>4.8123999999999997E-3</v>
+        <v>1.0019699999999999E-2</v>
       </c>
       <c r="W18">
-        <v>2.7819699999999999E-2</v>
+        <v>3.1512199999999997E-2</v>
       </c>
       <c r="X18">
-        <v>2.1110799999999999E-2</v>
+        <v>2.7052099999999999E-2</v>
       </c>
       <c r="Y18">
-        <v>5.5510900000000002E-2</v>
+        <v>6.0557199999999999E-2</v>
       </c>
       <c r="Z18">
-        <v>2.90523E-2</v>
+        <v>3.4375500000000003E-2</v>
       </c>
       <c r="AA18">
-        <v>7.2845199999999999E-2</v>
+        <v>8.1650899999999998E-2</v>
       </c>
       <c r="AB18">
-        <v>2.2410900000000001E-2</v>
+        <v>2.7579599999999999E-2</v>
       </c>
       <c r="AC18">
-        <v>8.0230599999999999E-2</v>
+        <v>8.54549E-2</v>
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.2">
@@ -2655,82 +2655,82 @@
         <v>46</v>
       </c>
       <c r="D19">
-        <v>2.9042800000000001E-2</v>
+        <v>2.9100999999999998E-2</v>
       </c>
       <c r="E19">
-        <v>6.3022300000000003E-2</v>
+        <v>6.3712099999999994E-2</v>
       </c>
       <c r="F19">
-        <v>7.2522799999999998E-2</v>
+        <v>7.6365600000000006E-2</v>
       </c>
       <c r="G19">
-        <v>6.2130299999999999E-2</v>
+        <v>5.9797999999999997E-2</v>
       </c>
       <c r="H19">
-        <v>4.9716900000000001E-2</v>
+        <v>5.2300600000000003E-2</v>
       </c>
       <c r="I19">
-        <v>-4.8672100000000003E-2</v>
+        <v>-5.5065900000000001E-2</v>
       </c>
       <c r="J19">
-        <v>-1.3428000000000001E-2</v>
+        <v>-2.48939E-2</v>
       </c>
       <c r="K19">
-        <v>-1.00067E-2</v>
+        <v>-1.0065299999999999E-2</v>
       </c>
       <c r="L19">
-        <v>-3.0447599999999998E-2</v>
+        <v>-3.2390799999999997E-2</v>
       </c>
       <c r="M19">
-        <v>-2.2331E-2</v>
+        <v>-3.0116E-2</v>
       </c>
       <c r="N19">
-        <v>-5.8311599999999998E-2</v>
+        <v>-6.9094500000000003E-2</v>
       </c>
       <c r="O19">
-        <v>-6.9763099999999995E-2</v>
+        <v>-6.8658499999999997E-2</v>
       </c>
       <c r="P19">
-        <v>7.7945200000000006E-2</v>
+        <v>7.6458799999999993E-2</v>
       </c>
       <c r="Q19">
-        <v>3.4464500000000002E-2</v>
+        <v>2.33879E-2</v>
       </c>
       <c r="R19">
-        <v>-0.1266158</v>
+        <v>-0.1422079</v>
       </c>
       <c r="S19">
-        <v>-0.1118198</v>
+        <v>-0.1273878</v>
       </c>
       <c r="T19">
-        <v>-0.12628610000000001</v>
+        <v>-0.14064289999999999</v>
       </c>
       <c r="U19" t="s">
         <v>29</v>
       </c>
       <c r="V19">
-        <v>1.9969299999999999E-2</v>
+        <v>2.7261199999999999E-2</v>
       </c>
       <c r="W19">
-        <v>-2.3614400000000001E-2</v>
+        <v>-2.7075800000000001E-2</v>
       </c>
       <c r="X19">
-        <v>-1.40447E-2</v>
+        <v>-1.35049E-2</v>
       </c>
       <c r="Y19">
-        <v>-3.90287E-2</v>
+        <v>-4.5783200000000003E-2</v>
       </c>
       <c r="Z19">
-        <v>-6.1033299999999999E-2</v>
+        <v>-7.1115800000000007E-2</v>
       </c>
       <c r="AA19">
-        <v>-2.76507E-2</v>
+        <v>-2.8861999999999999E-2</v>
       </c>
       <c r="AB19">
-        <v>-0.16555410000000001</v>
+        <v>-0.1829749</v>
       </c>
       <c r="AC19">
-        <v>0.16223679999999999</v>
+        <v>0.16782620000000001</v>
       </c>
     </row>
     <row r="20" spans="1:29" x14ac:dyDescent="0.2">
@@ -2744,254 +2744,260 @@
         <v>47</v>
       </c>
       <c r="D20">
-        <v>-9.4508700000000001E-2</v>
+        <v>-0.1016707</v>
       </c>
       <c r="E20">
-        <v>-7.8085100000000005E-2</v>
+        <v>-8.6318199999999998E-2</v>
       </c>
       <c r="F20">
-        <v>-8.6338600000000001E-2</v>
+        <v>-8.9220099999999997E-2</v>
       </c>
       <c r="G20">
-        <v>-7.2250099999999998E-2</v>
+        <v>-7.3216199999999995E-2</v>
       </c>
       <c r="H20">
-        <v>-9.0012900000000007E-2</v>
+        <v>-9.3107899999999993E-2</v>
       </c>
       <c r="I20">
-        <v>2.6221999999999999E-3</v>
+        <v>-5.4361000000000001E-3</v>
       </c>
       <c r="J20">
-        <v>3.2216700000000001E-2</v>
+        <v>2.87952E-2</v>
       </c>
       <c r="K20">
-        <v>2.4386000000000001E-2</v>
+        <v>3.3097300000000003E-2</v>
       </c>
       <c r="L20">
-        <v>3.5051100000000002E-2</v>
+        <v>4.9674099999999999E-2</v>
       </c>
       <c r="M20">
-        <v>2.89448E-2</v>
+        <v>2.7286600000000001E-2</v>
       </c>
       <c r="N20">
-        <v>3.0135100000000001E-2</v>
+        <v>2.1241900000000001E-2</v>
       </c>
       <c r="O20">
-        <v>9.0190800000000002E-2</v>
+        <v>0.1038253</v>
       </c>
       <c r="P20">
-        <v>6.7208699999999996E-2</v>
+        <v>6.57552E-2</v>
       </c>
       <c r="Q20">
-        <v>-0.16384689999999999</v>
+        <v>-0.17148160000000001</v>
       </c>
       <c r="R20">
-        <v>-0.2094077</v>
+        <v>-0.2298616</v>
       </c>
       <c r="S20">
-        <v>-0.19250300000000001</v>
+        <v>-0.2006356</v>
       </c>
       <c r="T20">
-        <v>-0.24159040000000001</v>
+        <v>-0.26479259999999999</v>
       </c>
       <c r="U20">
-        <v>-0.44774170000000002</v>
+        <v>-0.4904734</v>
       </c>
       <c r="V20" t="s">
         <v>29</v>
       </c>
       <c r="W20">
-        <v>-0.89722769999999996</v>
+        <v>-0.9631419</v>
       </c>
       <c r="X20">
-        <v>-0.85261160000000003</v>
+        <v>-0.91302470000000002</v>
       </c>
       <c r="Y20">
-        <v>-0.22900760000000001</v>
+        <v>-0.246918</v>
       </c>
       <c r="Z20">
-        <v>-0.19825880000000001</v>
+        <v>-0.21590000000000001</v>
       </c>
       <c r="AA20">
-        <v>-0.36590850000000003</v>
+        <v>-0.3995785</v>
       </c>
       <c r="AB20">
-        <v>-0.28378949999999997</v>
+        <v>-0.30993130000000002</v>
       </c>
       <c r="AC20">
-        <v>-5.7044299999999999E-2</v>
+        <v>-6.77981E-2</v>
       </c>
     </row>
     <row r="21" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2743</v>
       </c>
+      <c r="B21" t="s">
+        <v>61</v>
+      </c>
       <c r="C21" t="s">
         <v>48</v>
       </c>
       <c r="D21">
-        <v>-0.11375250000000001</v>
+        <v>-0.12096229999999999</v>
       </c>
       <c r="E21">
-        <v>-0.17011129999999999</v>
+        <v>-0.1866051</v>
       </c>
       <c r="F21">
-        <v>-0.15169959999999999</v>
+        <v>-0.15239040000000001</v>
       </c>
       <c r="G21">
-        <v>-0.1347748</v>
+        <v>-0.1383423</v>
       </c>
       <c r="H21">
-        <v>-0.1549769</v>
+        <v>-0.1594719</v>
       </c>
       <c r="I21">
-        <v>2.1324800000000001E-2</v>
+        <v>1.0721899999999999E-2</v>
       </c>
       <c r="J21">
-        <v>-4.6010200000000001E-2</v>
+        <v>-5.8843399999999997E-2</v>
       </c>
       <c r="K21">
-        <v>-0.1147339</v>
+        <v>-0.12122280000000001</v>
       </c>
       <c r="L21">
-        <v>-0.1063545</v>
+        <v>-0.1231661</v>
       </c>
       <c r="M21">
-        <v>3.6676599999999997E-2</v>
+        <v>2.2729599999999999E-2</v>
       </c>
       <c r="N21">
-        <v>1.06543E-2</v>
+        <v>2.7261E-3</v>
       </c>
       <c r="O21">
-        <v>3.2481299999999998E-2</v>
+        <v>2.45328E-2</v>
       </c>
       <c r="P21">
-        <v>5.0820400000000002E-2</v>
+        <v>4.1152099999999997E-2</v>
       </c>
       <c r="Q21">
-        <v>-7.0741299999999993E-2</v>
+        <v>-6.8862900000000005E-2</v>
       </c>
       <c r="R21">
-        <v>-0.226387</v>
+        <v>-0.24845790000000001</v>
       </c>
       <c r="S21">
-        <v>-0.19692889999999999</v>
+        <v>-0.22383910000000001</v>
       </c>
       <c r="T21">
-        <v>-0.220827</v>
+        <v>-0.24072479999999999</v>
       </c>
       <c r="U21">
-        <v>-0.1921947</v>
+        <v>-0.2187827</v>
       </c>
       <c r="V21">
-        <v>-0.27020460000000002</v>
+        <v>-0.28777390000000003</v>
       </c>
       <c r="W21" t="s">
         <v>29</v>
       </c>
       <c r="X21">
-        <v>-0.59966580000000003</v>
+        <v>-0.64620960000000005</v>
       </c>
       <c r="Y21">
-        <v>-0.23211789999999999</v>
+        <v>-0.26096740000000002</v>
       </c>
       <c r="Z21">
-        <v>-0.21556030000000001</v>
+        <v>-0.24096670000000001</v>
       </c>
       <c r="AA21">
-        <v>-0.1326861</v>
+        <v>-0.15408050000000001</v>
       </c>
       <c r="AB21">
-        <v>-0.1891159</v>
+        <v>-0.2115467</v>
       </c>
       <c r="AC21">
-        <v>6.5106399999999995E-2</v>
+        <v>6.8211800000000003E-2</v>
       </c>
     </row>
     <row r="22" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2846</v>
       </c>
+      <c r="B22" t="s">
+        <v>61</v>
+      </c>
       <c r="C22" t="s">
         <v>49</v>
       </c>
       <c r="D22">
-        <v>-2.1559100000000001E-2</v>
+        <v>-1.52249E-2</v>
       </c>
       <c r="E22">
-        <v>-8.0682799999999999E-2</v>
+        <v>-7.0746400000000001E-2</v>
       </c>
       <c r="F22">
-        <v>-9.16772E-2</v>
+        <v>-9.5175999999999997E-2</v>
       </c>
       <c r="G22">
-        <v>-6.79559E-2</v>
+        <v>-7.7774899999999994E-2</v>
       </c>
       <c r="H22">
-        <v>-6.9055500000000006E-2</v>
+        <v>-7.3658199999999993E-2</v>
       </c>
       <c r="I22">
-        <v>9.4363799999999998E-2</v>
+        <v>0.1030097</v>
       </c>
       <c r="J22">
-        <v>6.69207E-2</v>
+        <v>7.2478500000000001E-2</v>
       </c>
       <c r="K22">
-        <v>9.9497799999999997E-2</v>
+        <v>0.10043340000000001</v>
       </c>
       <c r="L22">
-        <v>4.3229299999999998E-2</v>
+        <v>4.8570700000000001E-2</v>
       </c>
       <c r="M22">
-        <v>0.13700560000000001</v>
+        <v>0.14564050000000001</v>
       </c>
       <c r="N22">
-        <v>0.12622079999999999</v>
+        <v>0.13208429999999999</v>
       </c>
       <c r="O22">
-        <v>0.1327942</v>
+        <v>0.1241216</v>
       </c>
       <c r="P22">
-        <v>0.1523052</v>
+        <v>0.15839239999999999</v>
       </c>
       <c r="Q22">
-        <v>-5.6067000000000001E-3</v>
+        <v>-6.2835E-3</v>
       </c>
       <c r="R22">
-        <v>-0.15616459999999999</v>
+        <v>-0.17155090000000001</v>
       </c>
       <c r="S22">
-        <v>-0.1278164</v>
+        <v>-0.13910220000000001</v>
       </c>
       <c r="T22">
-        <v>-0.126309</v>
+        <v>-0.14477760000000001</v>
       </c>
       <c r="U22">
-        <v>-0.16200120000000001</v>
+        <v>-0.17530409999999999</v>
       </c>
       <c r="V22">
-        <v>-0.41428090000000001</v>
+        <v>-0.44567479999999998</v>
       </c>
       <c r="W22">
-        <v>-0.75104130000000002</v>
+        <v>-0.81240599999999996</v>
       </c>
       <c r="X22" t="s">
         <v>29</v>
       </c>
       <c r="Y22">
-        <v>-0.15384429999999999</v>
+        <v>-0.17213249999999999</v>
       </c>
       <c r="Z22">
-        <v>-0.1252201</v>
+        <v>-0.13812350000000001</v>
       </c>
       <c r="AA22">
-        <v>-6.2148999999999998E-3</v>
+        <v>-1.5285200000000001E-2</v>
       </c>
       <c r="AB22">
-        <v>-0.1520523</v>
+        <v>-0.17129849999999999</v>
       </c>
       <c r="AC22">
-        <v>7.3514800000000005E-2</v>
+        <v>8.7348200000000001E-2</v>
       </c>
     </row>
     <row r="23" spans="1:29" x14ac:dyDescent="0.2">
@@ -3005,82 +3011,82 @@
         <v>50</v>
       </c>
       <c r="D23">
-        <v>9.9588999999999997E-2</v>
+        <v>0.106444</v>
       </c>
       <c r="E23">
-        <v>0.1415582</v>
+        <v>0.1552277</v>
       </c>
       <c r="F23">
-        <v>0.1423798</v>
+        <v>0.15234339999999999</v>
       </c>
       <c r="G23">
-        <v>0.1208794</v>
+        <v>0.12995809999999999</v>
       </c>
       <c r="H23">
-        <v>0.11528239999999999</v>
+        <v>0.1254846</v>
       </c>
       <c r="I23">
-        <v>5.1289399999999999E-2</v>
+        <v>5.5235600000000003E-2</v>
       </c>
       <c r="J23">
-        <v>2.8321699999999998E-2</v>
+        <v>3.03965E-2</v>
       </c>
       <c r="K23">
-        <v>0.17396809999999999</v>
+        <v>0.18354280000000001</v>
       </c>
       <c r="L23">
-        <v>0.16275990000000001</v>
+        <v>0.17340030000000001</v>
       </c>
       <c r="M23">
-        <v>-6.2991999999999996E-3</v>
+        <v>-5.0393E-3</v>
       </c>
       <c r="N23">
-        <v>2.9161E-3</v>
+        <v>4.6809E-3</v>
       </c>
       <c r="O23">
-        <v>3.8366699999999997E-2</v>
+        <v>4.6049399999999997E-2</v>
       </c>
       <c r="P23">
-        <v>8.9915900000000007E-2</v>
+        <v>9.9957500000000005E-2</v>
       </c>
       <c r="Q23">
-        <v>5.2774799999999997E-2</v>
+        <v>5.6828900000000002E-2</v>
       </c>
       <c r="R23">
-        <v>0.14634839999999999</v>
+        <v>0.15924250000000001</v>
       </c>
       <c r="S23">
-        <v>0.15728429999999999</v>
+        <v>0.1670508</v>
       </c>
       <c r="T23">
-        <v>0.1272636</v>
+        <v>0.1363278</v>
       </c>
       <c r="U23">
-        <v>0.11763170000000001</v>
+        <v>0.12699759999999999</v>
       </c>
       <c r="V23">
-        <v>0.1310241</v>
+        <v>0.13852149999999999</v>
       </c>
       <c r="W23">
-        <v>0.1196311</v>
+        <v>0.12908</v>
       </c>
       <c r="X23">
-        <v>0.12649379999999999</v>
+        <v>0.13545380000000001</v>
       </c>
       <c r="Y23" t="s">
         <v>29</v>
       </c>
       <c r="Z23">
-        <v>-2.8717800000000002E-2</v>
+        <v>-2.7662099999999998E-2</v>
       </c>
       <c r="AA23">
-        <v>5.6491399999999997E-2</v>
+        <v>6.24153E-2</v>
       </c>
       <c r="AB23">
-        <v>3.0349399999999999E-2</v>
+        <v>3.5907700000000001E-2</v>
       </c>
       <c r="AC23">
-        <v>7.5273999999999994E-2</v>
+        <v>8.2572499999999993E-2</v>
       </c>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.2">
@@ -3094,82 +3100,82 @@
         <v>51</v>
       </c>
       <c r="D24">
-        <v>5.2027799999999999E-2</v>
+        <v>5.7163100000000001E-2</v>
       </c>
       <c r="E24">
-        <v>0.13387060000000001</v>
+        <v>0.1410534</v>
       </c>
       <c r="F24">
-        <v>0.11292770000000001</v>
+        <v>0.1178756</v>
       </c>
       <c r="G24">
-        <v>0.1193337</v>
+        <v>0.1283213</v>
       </c>
       <c r="H24">
-        <v>9.1103900000000002E-2</v>
+        <v>9.8509299999999994E-2</v>
       </c>
       <c r="I24">
-        <v>1.7196099999999999E-2</v>
+        <v>1.3640899999999999E-2</v>
       </c>
       <c r="J24">
-        <v>8.1922000000000002E-3</v>
+        <v>3.2152999999999999E-3</v>
       </c>
       <c r="K24">
-        <v>0.1329689</v>
+        <v>0.1385343</v>
       </c>
       <c r="L24">
-        <v>0.1333482</v>
+        <v>0.14123849999999999</v>
       </c>
       <c r="M24">
-        <v>-3.3819299999999997E-2</v>
+        <v>-4.0219299999999999E-2</v>
       </c>
       <c r="N24">
-        <v>3.75406E-2</v>
+        <v>4.4445800000000001E-2</v>
       </c>
       <c r="O24">
-        <v>4.55693E-2</v>
+        <v>4.2355299999999999E-2</v>
       </c>
       <c r="P24">
-        <v>7.4381000000000003E-2</v>
+        <v>7.7409199999999997E-2</v>
       </c>
       <c r="Q24">
-        <v>4.4436999999999997E-2</v>
+        <v>4.7918099999999998E-2</v>
       </c>
       <c r="R24">
-        <v>0.13996040000000001</v>
+        <v>0.15163399999999999</v>
       </c>
       <c r="S24">
-        <v>0.15679789999999999</v>
+        <v>0.17148669999999999</v>
       </c>
       <c r="T24">
-        <v>0.12509149999999999</v>
+        <v>0.13530829999999999</v>
       </c>
       <c r="U24">
-        <v>0.14237549999999999</v>
+        <v>0.1504461</v>
       </c>
       <c r="V24">
-        <v>0.16801920000000001</v>
+        <v>0.18059939999999999</v>
       </c>
       <c r="W24">
-        <v>0.1510367</v>
+        <v>0.16125059999999999</v>
       </c>
       <c r="X24">
-        <v>0.1561767</v>
+        <v>0.16672090000000001</v>
       </c>
       <c r="Y24">
-        <v>1.2315100000000001E-2</v>
+        <v>4.6414000000000004E-3</v>
       </c>
       <c r="Z24" t="s">
         <v>29</v>
       </c>
       <c r="AA24">
-        <v>0.1084305</v>
+        <v>0.1126841</v>
       </c>
       <c r="AB24">
-        <v>0.1023251</v>
+        <v>0.1076545</v>
       </c>
       <c r="AC24">
-        <v>6.8395999999999998E-2</v>
+        <v>6.8432400000000004E-2</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.2">
@@ -3183,82 +3189,82 @@
         <v>52</v>
       </c>
       <c r="D25">
-        <v>-0.12311279999999999</v>
+        <v>-0.138184</v>
       </c>
       <c r="E25">
-        <v>-0.12560399999999999</v>
+        <v>-0.14453189999999999</v>
       </c>
       <c r="F25">
-        <v>-0.1766084</v>
+        <v>-0.19815720000000001</v>
       </c>
       <c r="G25">
-        <v>-0.18329010000000001</v>
+        <v>-0.20452670000000001</v>
       </c>
       <c r="H25">
-        <v>-0.2108177</v>
+        <v>-0.23859359999999999</v>
       </c>
       <c r="I25">
-        <v>-0.120875</v>
+        <v>-0.13778799999999999</v>
       </c>
       <c r="J25">
-        <v>-0.1760784</v>
+        <v>-0.19770789999999999</v>
       </c>
       <c r="K25">
-        <v>-0.13739850000000001</v>
+        <v>-0.15322089999999999</v>
       </c>
       <c r="L25">
-        <v>-0.1471044</v>
+        <v>-0.1672614</v>
       </c>
       <c r="M25">
-        <v>-0.13406309999999999</v>
+        <v>-0.14142440000000001</v>
       </c>
       <c r="N25">
-        <v>-4.1832099999999997E-2</v>
+        <v>-4.8748300000000001E-2</v>
       </c>
       <c r="O25">
-        <v>-3.6790200000000002E-2</v>
+        <v>-4.6045700000000002E-2</v>
       </c>
       <c r="P25">
-        <v>-5.7368000000000002E-2</v>
+        <v>-6.5349900000000002E-2</v>
       </c>
       <c r="Q25">
-        <v>-4.6856000000000002E-2</v>
+        <v>-6.2033199999999997E-2</v>
       </c>
       <c r="R25">
-        <v>-6.4569399999999999E-2</v>
+        <v>-8.1351900000000005E-2</v>
       </c>
       <c r="S25">
-        <v>-5.9445199999999997E-2</v>
+        <v>-7.7615900000000002E-2</v>
       </c>
       <c r="T25">
-        <v>-7.5845899999999994E-2</v>
+        <v>-9.4297900000000004E-2</v>
       </c>
       <c r="U25">
-        <v>-0.27724700000000002</v>
+        <v>-0.30793569999999998</v>
       </c>
       <c r="V25">
-        <v>-0.14041590000000001</v>
+        <v>-0.16600889999999999</v>
       </c>
       <c r="W25">
-        <v>-0.17172280000000001</v>
+        <v>-0.19000700000000001</v>
       </c>
       <c r="X25">
-        <v>-9.2839900000000003E-2</v>
+        <v>-0.1075612</v>
       </c>
       <c r="Y25">
-        <v>-0.19539329999999999</v>
+        <v>-0.2241215</v>
       </c>
       <c r="Z25">
-        <v>-0.2041721</v>
+        <v>-0.23007639999999999</v>
       </c>
       <c r="AA25" t="s">
         <v>29</v>
       </c>
       <c r="AB25">
-        <v>-0.36254249999999999</v>
+        <v>-0.40342470000000002</v>
       </c>
       <c r="AC25">
-        <v>-0.22726589999999999</v>
+        <v>-0.25495859999999998</v>
       </c>
     </row>
     <row r="26" spans="1:29" x14ac:dyDescent="0.2">
@@ -3269,82 +3275,82 @@
         <v>53</v>
       </c>
       <c r="D26">
-        <v>5.5080299999999999E-2</v>
+        <v>5.8304300000000003E-2</v>
       </c>
       <c r="E26">
-        <v>4.9326200000000001E-2</v>
+        <v>5.1789200000000001E-2</v>
       </c>
       <c r="F26">
-        <v>0.1307403</v>
+        <v>0.14078660000000001</v>
       </c>
       <c r="G26">
-        <v>9.7190700000000005E-2</v>
+        <v>0.1029268</v>
       </c>
       <c r="H26">
-        <v>8.6851300000000006E-2</v>
+        <v>9.3965699999999999E-2</v>
       </c>
       <c r="I26">
-        <v>0.28180100000000002</v>
+        <v>0.29966690000000001</v>
       </c>
       <c r="J26">
-        <v>0.28404740000000001</v>
+        <v>0.29805520000000002</v>
       </c>
       <c r="K26">
-        <v>-1.9813999999999998E-2</v>
+        <v>-2.2192199999999999E-2</v>
       </c>
       <c r="L26">
-        <v>-1.6871000000000001E-2</v>
+        <v>-1.2263E-2</v>
       </c>
       <c r="M26">
-        <v>0.27319510000000002</v>
+        <v>0.29983769999999998</v>
       </c>
       <c r="N26">
-        <v>0.1899988</v>
+        <v>0.2061598</v>
       </c>
       <c r="O26">
-        <v>0.2066963</v>
+        <v>0.2225306</v>
       </c>
       <c r="P26">
-        <v>0.12559699999999999</v>
+        <v>0.13506870000000001</v>
       </c>
       <c r="Q26">
-        <v>0.1034738</v>
+        <v>0.1172574</v>
       </c>
       <c r="R26">
-        <v>5.6244000000000002E-2</v>
+        <v>6.2525700000000003E-2</v>
       </c>
       <c r="S26">
-        <v>5.85578E-2</v>
+        <v>6.5854899999999994E-2</v>
       </c>
       <c r="T26">
-        <v>5.7823899999999998E-2</v>
+        <v>5.9068700000000002E-2</v>
       </c>
       <c r="U26">
-        <v>0.14910409999999999</v>
+        <v>0.1655394</v>
       </c>
       <c r="V26">
-        <v>0.31327640000000001</v>
+        <v>0.33812589999999998</v>
       </c>
       <c r="W26">
-        <v>0.2316558</v>
+        <v>0.24945149999999999</v>
       </c>
       <c r="X26">
-        <v>0.23188249999999999</v>
+        <v>0.24959410000000001</v>
       </c>
       <c r="Y26">
-        <v>3.47786E-2</v>
+        <v>3.4750799999999998E-2</v>
       </c>
       <c r="Z26">
-        <v>2.2808100000000001E-2</v>
+        <v>2.22154E-2</v>
       </c>
       <c r="AA26">
-        <v>0.16495370000000001</v>
+        <v>0.1827819</v>
       </c>
       <c r="AB26" t="s">
         <v>29</v>
       </c>
       <c r="AC26">
-        <v>0.26450849999999998</v>
+        <v>0.28078760000000003</v>
       </c>
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.2">
@@ -3355,79 +3361,79 @@
         <v>54</v>
       </c>
       <c r="D27">
-        <v>-6.7889999999999999E-3</v>
+        <v>-7.6845999999999998E-3</v>
       </c>
       <c r="E27">
-        <v>0.23891470000000001</v>
+        <v>0.25675419999999999</v>
       </c>
       <c r="F27">
-        <v>-6.4600500000000005E-2</v>
+        <v>-6.4260600000000001E-2</v>
       </c>
       <c r="G27">
-        <v>-3.4173599999999998E-2</v>
+        <v>-3.6928799999999998E-2</v>
       </c>
       <c r="H27">
-        <v>-5.9354999999999998E-3</v>
+        <v>-7.7222999999999997E-3</v>
       </c>
       <c r="I27">
-        <v>-5.9044699999999999E-2</v>
+        <v>-6.2206299999999999E-2</v>
       </c>
       <c r="J27">
-        <v>3.948E-4</v>
+        <v>-2.0018000000000002E-3</v>
       </c>
       <c r="K27">
-        <v>-0.12792529999999999</v>
+        <v>-0.1318397</v>
       </c>
       <c r="L27">
-        <v>-0.1004617</v>
+        <v>-0.1142746</v>
       </c>
       <c r="M27">
-        <v>-3.3342299999999998E-2</v>
+        <v>-3.3419200000000003E-2</v>
       </c>
       <c r="N27">
-        <v>-1.0843200000000001E-2</v>
+        <v>-1.14003E-2</v>
       </c>
       <c r="O27">
-        <v>-3.0245899999999999E-2</v>
+        <v>-3.5143199999999999E-2</v>
       </c>
       <c r="P27">
-        <v>-0.10880570000000001</v>
+        <v>-0.11805789999999999</v>
       </c>
       <c r="Q27">
-        <v>6.1485999999999997E-3</v>
+        <v>2.0683199999999999E-2</v>
       </c>
       <c r="R27">
-        <v>5.6860000000000005E-4</v>
+        <v>1.04934E-2</v>
       </c>
       <c r="S27">
-        <v>-6.6944400000000001E-2</v>
+        <v>-6.0326999999999999E-2</v>
       </c>
       <c r="T27">
-        <v>1.6930500000000001E-2</v>
+        <v>2.3033000000000001E-2</v>
       </c>
       <c r="U27">
-        <v>-7.33399E-2</v>
+        <v>-7.7376600000000004E-2</v>
       </c>
       <c r="V27">
-        <v>-7.9747299999999993E-2</v>
+        <v>-9.0441300000000002E-2</v>
       </c>
       <c r="W27">
-        <v>-0.1017729</v>
+        <v>-0.1109682</v>
       </c>
       <c r="X27">
-        <v>-0.1143967</v>
+        <v>-0.1229502</v>
       </c>
       <c r="Y27">
-        <v>-3.4099200000000003E-2</v>
+        <v>-3.6686200000000002E-2</v>
       </c>
       <c r="Z27">
-        <v>-6.3894500000000007E-2</v>
+        <v>-6.14665E-2</v>
       </c>
       <c r="AA27">
-        <v>-0.1738498</v>
+        <v>-0.18654219999999999</v>
       </c>
       <c r="AB27">
-        <v>-6.7741200000000001E-2</v>
+        <v>-7.3865600000000003E-2</v>
       </c>
       <c r="AC27" t="s">
         <v>29</v>
@@ -3437,12 +3443,12 @@
   <conditionalFormatting sqref="D2:AC27">
     <cfRule type="colorScale" priority="1">
       <colorScale>
-        <cfvo type="num" val="-0.3"/>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0.3"/>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
         <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>

</xml_diff>